<commit_message>
updated designs sent to khu
</commit_message>
<xml_diff>
--- a/inventory_khu/Inventory_final.xlsx
+++ b/inventory_khu/Inventory_final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wkdqh\Dropbox\패밀리룸\촉매반응연구실\2.연구\연구 프로젝트 결과\박민철\13. 안광노 박사님\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{085C51B6-4C68-4B56-92B9-B72DBEA1FC0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1634EA3B-E33F-4EBC-8CB1-D9B84CA5F0D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2970" windowWidth="29040" windowHeight="15720" tabRatio="814" activeTab="1" xr2:uid="{BA5EE998-393C-4222-9A45-0D82231A5A27}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="814" activeTab="3" xr2:uid="{BA5EE998-393C-4222-9A45-0D82231A5A27}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="8" r:id="rId1"/>
@@ -215,7 +215,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="204">
   <si>
     <t>모델명</t>
   </si>
@@ -7998,6 +7998,34 @@
       </rPr>
       <t>있도록 개선되면 좋을 것 같습니다.</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">호환가능 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>module</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UV-150, manual photoreactor</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -8480,7 +8508,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -8652,6 +8680,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -8676,7 +8707,19 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -8685,37 +8728,25 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9081,30 +9112,30 @@
       </c>
     </row>
     <row r="6" spans="2:11" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="B6" s="57" t="s">
+      <c r="B6" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="C6" s="57"/>
-      <c r="D6" s="57"/>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57"/>
-      <c r="H6" s="57"/>
-      <c r="I6" s="57"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="58"/>
+      <c r="I6" s="58"/>
       <c r="J6" s="40"/>
       <c r="K6" s="40"/>
     </row>
     <row r="7" spans="2:11" ht="20.65" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="B7" s="57" t="s">
+      <c r="B7" s="58" t="s">
         <v>124</v>
       </c>
-      <c r="C7" s="57"/>
-      <c r="D7" s="57"/>
-      <c r="E7" s="57"/>
-      <c r="F7" s="57"/>
-      <c r="G7" s="57"/>
-      <c r="H7" s="57"/>
-      <c r="I7" s="57"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="58"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="58"/>
+      <c r="I7" s="58"/>
       <c r="J7" s="40"/>
       <c r="K7" s="40"/>
     </row>
@@ -9119,76 +9150,76 @@
       <c r="I8" s="41"/>
     </row>
     <row r="9" spans="2:11" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="B9" s="58" t="s">
+      <c r="B9" s="59" t="s">
         <v>123</v>
       </c>
-      <c r="C9" s="58"/>
-      <c r="D9" s="58"/>
-      <c r="E9" s="58"/>
-      <c r="F9" s="58"/>
-      <c r="G9" s="58"/>
-      <c r="H9" s="58"/>
-      <c r="I9" s="58"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="59"/>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.6">
-      <c r="B10" s="59" t="s">
+      <c r="B10" s="60" t="s">
         <v>125</v>
       </c>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="59"/>
-      <c r="I10" s="59"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60"/>
+      <c r="H10" s="60"/>
+      <c r="I10" s="60"/>
     </row>
     <row r="12" spans="2:11" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="B12" s="58" t="s">
+      <c r="B12" s="59" t="s">
         <v>126</v>
       </c>
-      <c r="C12" s="58"/>
-      <c r="D12" s="58"/>
-      <c r="E12" s="58"/>
-      <c r="F12" s="58"/>
-      <c r="G12" s="58"/>
-      <c r="H12" s="58"/>
-      <c r="I12" s="58"/>
+      <c r="C12" s="59"/>
+      <c r="D12" s="59"/>
+      <c r="E12" s="59"/>
+      <c r="F12" s="59"/>
+      <c r="G12" s="59"/>
+      <c r="H12" s="59"/>
+      <c r="I12" s="59"/>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.6">
-      <c r="B13" s="59" t="s">
+      <c r="B13" s="60" t="s">
         <v>127</v>
       </c>
-      <c r="C13" s="59"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="59"/>
-      <c r="F13" s="59"/>
-      <c r="G13" s="59"/>
-      <c r="H13" s="59"/>
-      <c r="I13" s="59"/>
+      <c r="C13" s="60"/>
+      <c r="D13" s="60"/>
+      <c r="E13" s="60"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="60"/>
+      <c r="H13" s="60"/>
+      <c r="I13" s="60"/>
     </row>
     <row r="15" spans="2:11" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="B15" s="58" t="s">
+      <c r="B15" s="59" t="s">
         <v>182</v>
       </c>
-      <c r="C15" s="58"/>
-      <c r="D15" s="58"/>
-      <c r="E15" s="58"/>
-      <c r="F15" s="58"/>
-      <c r="G15" s="58"/>
-      <c r="H15" s="58"/>
-      <c r="I15" s="58"/>
+      <c r="C15" s="59"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="59"/>
+      <c r="F15" s="59"/>
+      <c r="G15" s="59"/>
+      <c r="H15" s="59"/>
+      <c r="I15" s="59"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.6">
-      <c r="B17" s="59" t="s">
+      <c r="B17" s="60" t="s">
         <v>183</v>
       </c>
-      <c r="C17" s="59"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="59"/>
-      <c r="F17" s="59"/>
-      <c r="G17" s="59"/>
-      <c r="H17" s="59"/>
-      <c r="I17" s="59"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="60"/>
+      <c r="G17" s="60"/>
+      <c r="H17" s="60"/>
+      <c r="I17" s="60"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.6">
       <c r="B19" s="36" t="s">
@@ -9537,29 +9568,29 @@
     </row>
     <row r="10" spans="1:11" ht="38.65" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B10" s="35"/>
-      <c r="C10" s="60" t="s">
+      <c r="C10" s="61" t="s">
         <v>187</v>
       </c>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
-      <c r="G10" s="60"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="60"/>
-      <c r="J10" s="60"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="61"/>
+      <c r="J10" s="61"/>
     </row>
     <row r="11" spans="1:11" ht="39.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B11" s="35"/>
-      <c r="C11" s="60" t="s">
+      <c r="C11" s="61" t="s">
         <v>201</v>
       </c>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-      <c r="J11" s="60"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
+      <c r="J11" s="61"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.6">
       <c r="H16" s="56"/>
@@ -9641,7 +9672,7 @@
       <c r="D3" s="8">
         <v>4.7</v>
       </c>
-      <c r="E3" s="61" t="s">
+      <c r="E3" s="62" t="s">
         <v>103</v>
       </c>
       <c r="F3" s="8">
@@ -9653,16 +9684,16 @@
       <c r="H3" s="8">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="I3" s="61" t="s">
+      <c r="I3" s="62" t="s">
         <v>115</v>
       </c>
-      <c r="J3" s="61">
+      <c r="J3" s="62">
         <v>999</v>
       </c>
       <c r="K3" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="L3" s="61" t="s">
+      <c r="L3" s="62" t="s">
         <v>27</v>
       </c>
       <c r="M3" s="33"/>
@@ -9677,7 +9708,7 @@
       <c r="D4" s="8">
         <v>9.6999999999999993</v>
       </c>
-      <c r="E4" s="61"/>
+      <c r="E4" s="62"/>
       <c r="F4" s="8">
         <v>1E-4</v>
       </c>
@@ -9687,12 +9718,12 @@
       <c r="H4" s="8">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="I4" s="61"/>
-      <c r="J4" s="61"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
       <c r="K4" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="L4" s="61"/>
+      <c r="L4" s="62"/>
       <c r="M4" s="33"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.6">
@@ -9705,7 +9736,7 @@
       <c r="D5" s="8">
         <v>12.48</v>
       </c>
-      <c r="E5" s="61"/>
+      <c r="E5" s="62"/>
       <c r="F5" s="8">
         <v>1E-4</v>
       </c>
@@ -9715,12 +9746,12 @@
       <c r="H5" s="8">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="I5" s="61"/>
-      <c r="J5" s="61"/>
+      <c r="I5" s="62"/>
+      <c r="J5" s="62"/>
       <c r="K5" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="L5" s="61"/>
+      <c r="L5" s="62"/>
       <c r="M5" s="33"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.6">
@@ -9733,7 +9764,7 @@
       <c r="D6" s="8">
         <v>15.89</v>
       </c>
-      <c r="E6" s="61"/>
+      <c r="E6" s="62"/>
       <c r="F6" s="8">
         <v>1E-4</v>
       </c>
@@ -9743,12 +9774,12 @@
       <c r="H6" s="8">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="I6" s="61"/>
-      <c r="J6" s="61"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="62"/>
       <c r="K6" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="L6" s="61"/>
+      <c r="L6" s="62"/>
       <c r="M6" s="33"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.6">
@@ -9761,7 +9792,7 @@
       <c r="D7" s="8">
         <v>20</v>
       </c>
-      <c r="E7" s="61"/>
+      <c r="E7" s="62"/>
       <c r="F7" s="8">
         <v>1E-4</v>
       </c>
@@ -9771,12 +9802,12 @@
       <c r="H7" s="8">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="I7" s="61"/>
-      <c r="J7" s="61"/>
+      <c r="I7" s="62"/>
+      <c r="J7" s="62"/>
       <c r="K7" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="L7" s="61"/>
+      <c r="L7" s="62"/>
       <c r="M7" s="33"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.6">
@@ -9789,7 +9820,7 @@
       <c r="D8" s="8">
         <v>7.29</v>
       </c>
-      <c r="E8" s="61" t="s">
+      <c r="E8" s="62" t="s">
         <v>113</v>
       </c>
       <c r="F8" s="8">
@@ -9801,7 +9832,7 @@
       <c r="H8" s="8">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="I8" s="62" t="s">
+      <c r="I8" s="63" t="s">
         <v>114</v>
       </c>
       <c r="J8" s="8">
@@ -9810,7 +9841,7 @@
       <c r="K8" s="51" t="s">
         <v>189</v>
       </c>
-      <c r="L8" s="61"/>
+      <c r="L8" s="62"/>
       <c r="M8" s="33"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.6">
@@ -9823,7 +9854,7 @@
       <c r="D9" s="8">
         <v>14.6</v>
       </c>
-      <c r="E9" s="61"/>
+      <c r="E9" s="62"/>
       <c r="F9" s="8">
         <v>1E-4</v>
       </c>
@@ -9833,14 +9864,14 @@
       <c r="H9" s="8">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="I9" s="63"/>
+      <c r="I9" s="64"/>
       <c r="J9" s="8">
         <v>2</v>
       </c>
       <c r="K9" s="51" t="s">
         <v>189</v>
       </c>
-      <c r="L9" s="61"/>
+      <c r="L9" s="62"/>
       <c r="M9" s="33"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.6">
@@ -9853,7 +9884,7 @@
       <c r="D10" s="51">
         <v>6.52</v>
       </c>
-      <c r="E10" s="61"/>
+      <c r="E10" s="62"/>
       <c r="F10" s="8">
         <v>0.02</v>
       </c>
@@ -9863,14 +9894,14 @@
       <c r="H10" s="8">
         <v>0.01</v>
       </c>
-      <c r="I10" s="63"/>
+      <c r="I10" s="64"/>
       <c r="J10" s="8">
         <v>4</v>
       </c>
       <c r="K10" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="L10" s="61" t="s">
+      <c r="L10" s="62" t="s">
         <v>21</v>
       </c>
       <c r="M10" s="33"/>
@@ -9885,7 +9916,7 @@
       <c r="D11" s="51">
         <v>14.6</v>
       </c>
-      <c r="E11" s="61"/>
+      <c r="E11" s="62"/>
       <c r="F11" s="8">
         <v>0.1</v>
       </c>
@@ -9895,14 +9926,14 @@
       <c r="H11" s="8">
         <v>0.1</v>
       </c>
-      <c r="I11" s="64"/>
+      <c r="I11" s="65"/>
       <c r="J11" s="8">
         <v>2</v>
       </c>
       <c r="K11" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="L11" s="61"/>
+      <c r="L11" s="62"/>
       <c r="M11" s="33"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.6">
@@ -9926,7 +9957,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F24C350A-89A2-414A-A488-36D2AC6D1085}">
-  <dimension ref="B2:K13"/>
+  <dimension ref="B2:L13"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="2" max="2" width="24" style="1" customWidth="1"/>
@@ -9938,10 +9969,11 @@
     <col min="8" max="8" width="18.875" style="1" customWidth="1"/>
     <col min="9" max="9" width="19.25" style="1" customWidth="1"/>
     <col min="10" max="10" width="21.125" customWidth="1"/>
-    <col min="11" max="11" width="44.625" customWidth="1"/>
+    <col min="11" max="11" width="24.0625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="44.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B2" s="10" t="s">
         <v>37</v>
       </c>
@@ -9969,11 +10001,14 @@
       <c r="J2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="11" t="s">
+      <c r="K2" s="34" t="s">
+        <v>202</v>
+      </c>
+      <c r="L2" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B3" s="51">
         <v>1</v>
       </c>
@@ -9983,10 +10018,10 @@
       <c r="D3" s="51">
         <v>2</v>
       </c>
-      <c r="E3" s="61">
+      <c r="E3" s="62">
         <v>1</v>
       </c>
-      <c r="F3" s="61">
+      <c r="F3" s="62">
         <v>1.6</v>
       </c>
       <c r="G3" s="51">
@@ -10001,9 +10036,12 @@
       <c r="J3" s="51">
         <v>34</v>
       </c>
-      <c r="K3" s="51"/>
+      <c r="K3" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L3" s="51"/>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B4" s="51">
         <v>2</v>
       </c>
@@ -10013,8 +10051,8 @@
       <c r="D4" s="51">
         <v>5</v>
       </c>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
       <c r="G4" s="51">
         <v>2</v>
       </c>
@@ -10027,9 +10065,12 @@
       <c r="J4" s="51">
         <v>34</v>
       </c>
-      <c r="K4" s="51"/>
+      <c r="K4" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L4" s="51"/>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B5" s="51">
         <v>3</v>
       </c>
@@ -10039,8 +10080,8 @@
       <c r="D5" s="51">
         <v>10</v>
       </c>
-      <c r="E5" s="61"/>
-      <c r="F5" s="61"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
       <c r="G5" s="51">
         <v>1</v>
       </c>
@@ -10053,9 +10094,12 @@
       <c r="J5" s="51">
         <v>34</v>
       </c>
-      <c r="K5" s="51"/>
+      <c r="K5" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L5" s="51"/>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B6" s="51">
         <v>5</v>
       </c>
@@ -10065,8 +10109,8 @@
       <c r="D6" s="51">
         <v>10</v>
       </c>
-      <c r="E6" s="61"/>
-      <c r="F6" s="61"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
       <c r="G6" s="51">
         <v>1</v>
       </c>
@@ -10079,9 +10123,12 @@
       <c r="J6" s="51">
         <v>34</v>
       </c>
-      <c r="K6" s="51"/>
+      <c r="K6" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L6" s="51"/>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B7" s="51">
         <v>6</v>
       </c>
@@ -10091,8 +10138,8 @@
       <c r="D7" s="51">
         <v>20</v>
       </c>
-      <c r="E7" s="61"/>
-      <c r="F7" s="61"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
       <c r="G7" s="51">
         <v>1</v>
       </c>
@@ -10105,9 +10152,12 @@
       <c r="J7" s="51">
         <v>34</v>
       </c>
-      <c r="K7" s="51"/>
+      <c r="K7" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L7" s="51"/>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B8" s="51">
         <v>7</v>
       </c>
@@ -10120,7 +10170,7 @@
       <c r="E8" s="51">
         <v>0.75</v>
       </c>
-      <c r="F8" s="61"/>
+      <c r="F8" s="62"/>
       <c r="G8" s="51">
         <v>1</v>
       </c>
@@ -10133,9 +10183,12 @@
       <c r="J8" s="51">
         <v>69</v>
       </c>
-      <c r="K8" s="51"/>
+      <c r="K8" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L8" s="51"/>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B9" s="51">
         <v>8</v>
       </c>
@@ -10145,10 +10198,10 @@
       <c r="D9" s="51" t="s">
         <v>192</v>
       </c>
-      <c r="E9" s="61">
+      <c r="E9" s="62">
         <v>0.5</v>
       </c>
-      <c r="F9" s="61"/>
+      <c r="F9" s="62"/>
       <c r="G9" s="51" t="s">
         <v>26</v>
       </c>
@@ -10161,11 +10214,14 @@
       <c r="J9" s="51">
         <v>138</v>
       </c>
-      <c r="K9" s="51" t="s">
+      <c r="K9" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L9" s="51" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B10" s="51">
         <v>9</v>
       </c>
@@ -10175,8 +10231,8 @@
       <c r="D10" s="51" t="s">
         <v>115</v>
       </c>
-      <c r="E10" s="61"/>
-      <c r="F10" s="61"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
       <c r="G10" s="51" t="s">
         <v>26</v>
       </c>
@@ -10189,11 +10245,14 @@
       <c r="J10" s="51">
         <v>138</v>
       </c>
-      <c r="K10" s="51" t="s">
+      <c r="K10" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L10" s="51" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B11" s="51">
         <v>9</v>
       </c>
@@ -10221,9 +10280,12 @@
       <c r="J11" s="51">
         <v>34</v>
       </c>
-      <c r="K11" s="51"/>
+      <c r="K11" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L11" s="51"/>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B12" s="51">
         <v>10</v>
       </c>
@@ -10249,9 +10311,12 @@
       <c r="J12" s="51">
         <v>34</v>
       </c>
-      <c r="K12" s="51"/>
+      <c r="K12" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L12" s="51"/>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.6">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.6">
       <c r="B13" s="51">
         <v>11</v>
       </c>
@@ -10279,7 +10344,10 @@
       <c r="J13" s="51">
         <v>34</v>
       </c>
-      <c r="K13" s="51" t="s">
+      <c r="K13" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L13" s="51" t="s">
         <v>195</v>
       </c>
     </row>
@@ -10368,13 +10436,13 @@
       </c>
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.6">
-      <c r="B3" s="66" t="s">
+      <c r="B3" s="71" t="s">
         <v>179</v>
       </c>
-      <c r="C3" s="61" t="s">
+      <c r="C3" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="68" t="s">
+      <c r="D3" s="74" t="s">
         <v>54</v>
       </c>
       <c r="E3" s="8" t="s">
@@ -10392,35 +10460,35 @@
       <c r="I3" s="8">
         <v>62</v>
       </c>
-      <c r="J3" s="61">
+      <c r="J3" s="62">
         <v>20</v>
       </c>
-      <c r="K3" s="61">
+      <c r="K3" s="62">
         <v>40</v>
       </c>
-      <c r="L3" s="61">
+      <c r="L3" s="62">
         <v>50</v>
       </c>
-      <c r="M3" s="61" t="s">
+      <c r="M3" s="62" t="s">
         <v>26</v>
       </c>
       <c r="N3" s="51">
         <v>2</v>
       </c>
-      <c r="O3" s="62">
+      <c r="O3" s="63">
         <v>1</v>
       </c>
-      <c r="P3" s="61" t="s">
+      <c r="P3" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="Q3" s="74" t="s">
+      <c r="Q3" s="66" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="4" spans="2:17" x14ac:dyDescent="0.6">
-      <c r="B4" s="66"/>
-      <c r="C4" s="61"/>
-      <c r="D4" s="68"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="74"/>
       <c r="E4" s="8" t="s">
         <v>56</v>
       </c>
@@ -10436,21 +10504,21 @@
       <c r="I4" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="J4" s="61"/>
-      <c r="K4" s="61"/>
-      <c r="L4" s="61"/>
-      <c r="M4" s="61"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="62"/>
+      <c r="L4" s="62"/>
+      <c r="M4" s="62"/>
       <c r="N4" s="51">
         <v>1</v>
       </c>
-      <c r="O4" s="63"/>
-      <c r="P4" s="61"/>
-      <c r="Q4" s="73"/>
+      <c r="O4" s="64"/>
+      <c r="P4" s="62"/>
+      <c r="Q4" s="67"/>
     </row>
     <row r="5" spans="2:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="B5" s="67"/>
-      <c r="C5" s="65"/>
-      <c r="D5" s="69"/>
+      <c r="B5" s="72"/>
+      <c r="C5" s="69"/>
+      <c r="D5" s="75"/>
       <c r="E5" s="24" t="s">
         <v>57</v>
       </c>
@@ -10466,25 +10534,25 @@
       <c r="I5" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="J5" s="65"/>
-      <c r="K5" s="65"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="65"/>
+      <c r="J5" s="69"/>
+      <c r="K5" s="69"/>
+      <c r="L5" s="69"/>
+      <c r="M5" s="69"/>
       <c r="N5" s="52">
         <v>1</v>
       </c>
-      <c r="O5" s="71"/>
-      <c r="P5" s="65"/>
-      <c r="Q5" s="73"/>
+      <c r="O5" s="76"/>
+      <c r="P5" s="69"/>
+      <c r="Q5" s="67"/>
     </row>
     <row r="6" spans="2:17" x14ac:dyDescent="0.6">
-      <c r="B6" s="78" t="s">
+      <c r="B6" s="77" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="78" t="s">
+      <c r="C6" s="77" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="78" t="s">
+      <c r="D6" s="77" t="s">
         <v>50</v>
       </c>
       <c r="E6" s="14" t="s">
@@ -10493,7 +10561,7 @@
       <c r="F6" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="72" t="s">
+      <c r="G6" s="78" t="s">
         <v>74</v>
       </c>
       <c r="H6" s="14" t="s">
@@ -10502,205 +10570,205 @@
       <c r="I6" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="J6" s="72">
+      <c r="J6" s="78">
         <v>10</v>
       </c>
-      <c r="K6" s="72">
+      <c r="K6" s="78">
         <v>25</v>
       </c>
-      <c r="L6" s="72">
+      <c r="L6" s="78">
         <v>80</v>
       </c>
-      <c r="M6" s="72">
+      <c r="M6" s="78">
         <v>1</v>
       </c>
       <c r="N6" s="53">
         <v>1</v>
       </c>
-      <c r="O6" s="72">
+      <c r="O6" s="78">
         <v>1</v>
       </c>
-      <c r="P6" s="72" t="s">
+      <c r="P6" s="78" t="s">
         <v>51</v>
       </c>
-      <c r="Q6" s="73"/>
+      <c r="Q6" s="67"/>
     </row>
     <row r="7" spans="2:17" x14ac:dyDescent="0.6">
-      <c r="B7" s="61"/>
-      <c r="C7" s="61"/>
-      <c r="D7" s="61"/>
+      <c r="B7" s="62"/>
+      <c r="C7" s="62"/>
+      <c r="D7" s="62"/>
       <c r="E7" s="8" t="s">
         <v>61</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="63"/>
+      <c r="G7" s="64"/>
       <c r="H7" s="8" t="s">
         <v>69</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="J7" s="63"/>
-      <c r="K7" s="63"/>
-      <c r="L7" s="63"/>
-      <c r="M7" s="63"/>
+      <c r="J7" s="64"/>
+      <c r="K7" s="64"/>
+      <c r="L7" s="64"/>
+      <c r="M7" s="64"/>
       <c r="N7" s="51">
         <v>1</v>
       </c>
-      <c r="O7" s="63"/>
-      <c r="P7" s="63"/>
-      <c r="Q7" s="73"/>
+      <c r="O7" s="64"/>
+      <c r="P7" s="64"/>
+      <c r="Q7" s="67"/>
     </row>
     <row r="8" spans="2:17" x14ac:dyDescent="0.6">
-      <c r="B8" s="61"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="61"/>
+      <c r="B8" s="62"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
       <c r="E8" s="8" t="s">
         <v>62</v>
       </c>
       <c r="F8" s="8">
         <v>396</v>
       </c>
-      <c r="G8" s="63"/>
+      <c r="G8" s="64"/>
       <c r="H8" s="8" t="s">
         <v>70</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="J8" s="63"/>
-      <c r="K8" s="63"/>
-      <c r="L8" s="63"/>
-      <c r="M8" s="63"/>
+      <c r="J8" s="64"/>
+      <c r="K8" s="64"/>
+      <c r="L8" s="64"/>
+      <c r="M8" s="64"/>
       <c r="N8" s="51">
         <v>1</v>
       </c>
-      <c r="O8" s="63"/>
-      <c r="P8" s="63"/>
-      <c r="Q8" s="73"/>
+      <c r="O8" s="64"/>
+      <c r="P8" s="64"/>
+      <c r="Q8" s="67"/>
     </row>
     <row r="9" spans="2:17" x14ac:dyDescent="0.6">
-      <c r="B9" s="61"/>
-      <c r="C9" s="61"/>
-      <c r="D9" s="61"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="62"/>
       <c r="E9" s="8" t="s">
         <v>63</v>
       </c>
       <c r="F9" s="8">
         <v>424</v>
       </c>
-      <c r="G9" s="63"/>
+      <c r="G9" s="64"/>
       <c r="H9" s="8" t="s">
         <v>71</v>
       </c>
       <c r="I9" s="8">
         <v>243</v>
       </c>
-      <c r="J9" s="63"/>
-      <c r="K9" s="63"/>
-      <c r="L9" s="63"/>
-      <c r="M9" s="63"/>
+      <c r="J9" s="64"/>
+      <c r="K9" s="64"/>
+      <c r="L9" s="64"/>
+      <c r="M9" s="64"/>
       <c r="N9" s="51">
         <v>1</v>
       </c>
-      <c r="O9" s="63"/>
-      <c r="P9" s="63"/>
-      <c r="Q9" s="73"/>
+      <c r="O9" s="64"/>
+      <c r="P9" s="64"/>
+      <c r="Q9" s="67"/>
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.6">
-      <c r="B10" s="61"/>
-      <c r="C10" s="61"/>
-      <c r="D10" s="61"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
       <c r="E10" s="8" t="s">
         <v>64</v>
       </c>
       <c r="F10" s="8">
         <v>450</v>
       </c>
-      <c r="G10" s="63"/>
+      <c r="G10" s="64"/>
       <c r="H10" s="8" t="s">
         <v>72</v>
       </c>
       <c r="I10" s="8">
         <v>355</v>
       </c>
-      <c r="J10" s="63"/>
-      <c r="K10" s="63"/>
-      <c r="L10" s="63"/>
-      <c r="M10" s="63"/>
+      <c r="J10" s="64"/>
+      <c r="K10" s="64"/>
+      <c r="L10" s="64"/>
+      <c r="M10" s="64"/>
       <c r="N10" s="51">
         <v>1</v>
       </c>
-      <c r="O10" s="63"/>
-      <c r="P10" s="63"/>
-      <c r="Q10" s="73"/>
+      <c r="O10" s="64"/>
+      <c r="P10" s="64"/>
+      <c r="Q10" s="67"/>
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.6">
-      <c r="B11" s="61"/>
-      <c r="C11" s="61"/>
-      <c r="D11" s="61"/>
+      <c r="B11" s="62"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
       <c r="E11" s="8" t="s">
         <v>65</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="63"/>
+      <c r="G11" s="64"/>
       <c r="H11" s="8" t="s">
         <v>72</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="J11" s="63"/>
-      <c r="K11" s="63"/>
-      <c r="L11" s="63"/>
-      <c r="M11" s="63"/>
+      <c r="J11" s="64"/>
+      <c r="K11" s="64"/>
+      <c r="L11" s="64"/>
+      <c r="M11" s="64"/>
       <c r="N11" s="51">
         <v>1</v>
       </c>
-      <c r="O11" s="63"/>
-      <c r="P11" s="63"/>
-      <c r="Q11" s="73"/>
+      <c r="O11" s="64"/>
+      <c r="P11" s="64"/>
+      <c r="Q11" s="67"/>
     </row>
     <row r="12" spans="2:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="B12" s="65"/>
-      <c r="C12" s="65"/>
-      <c r="D12" s="65"/>
+      <c r="B12" s="69"/>
+      <c r="C12" s="69"/>
+      <c r="D12" s="69"/>
       <c r="E12" s="52" t="s">
         <v>66</v>
       </c>
       <c r="F12" s="52">
         <v>533</v>
       </c>
-      <c r="G12" s="71"/>
+      <c r="G12" s="76"/>
       <c r="H12" s="52" t="s">
         <v>68</v>
       </c>
       <c r="I12" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="J12" s="71"/>
-      <c r="K12" s="71"/>
-      <c r="L12" s="71"/>
-      <c r="M12" s="71"/>
+      <c r="J12" s="76"/>
+      <c r="K12" s="76"/>
+      <c r="L12" s="76"/>
+      <c r="M12" s="76"/>
       <c r="N12" s="52">
         <v>1</v>
       </c>
-      <c r="O12" s="71"/>
-      <c r="P12" s="71"/>
-      <c r="Q12" s="73"/>
+      <c r="O12" s="76"/>
+      <c r="P12" s="76"/>
+      <c r="Q12" s="67"/>
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.6">
-      <c r="B13" s="76" t="s">
+      <c r="B13" s="70" t="s">
         <v>180</v>
       </c>
-      <c r="C13" s="64" t="s">
+      <c r="C13" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="77" t="s">
+      <c r="D13" s="73" t="s">
         <v>54</v>
       </c>
       <c r="E13" s="53" t="s">
@@ -10718,33 +10786,33 @@
       <c r="I13" s="53" t="s">
         <v>26</v>
       </c>
-      <c r="J13" s="64">
+      <c r="J13" s="65">
         <v>20</v>
       </c>
-      <c r="K13" s="64">
+      <c r="K13" s="65">
         <v>25</v>
       </c>
-      <c r="L13" s="64">
+      <c r="L13" s="65">
         <v>80</v>
       </c>
-      <c r="M13" s="64">
+      <c r="M13" s="65">
         <v>1</v>
       </c>
       <c r="N13" s="53">
         <v>2</v>
       </c>
-      <c r="O13" s="63">
+      <c r="O13" s="64">
         <v>1</v>
       </c>
-      <c r="P13" s="64" t="s">
+      <c r="P13" s="65" t="s">
         <v>181</v>
       </c>
-      <c r="Q13" s="73"/>
+      <c r="Q13" s="67"/>
     </row>
     <row r="14" spans="2:17" x14ac:dyDescent="0.6">
-      <c r="B14" s="66"/>
-      <c r="C14" s="61"/>
-      <c r="D14" s="68"/>
+      <c r="B14" s="71"/>
+      <c r="C14" s="62"/>
+      <c r="D14" s="74"/>
       <c r="E14" s="8" t="s">
         <v>56</v>
       </c>
@@ -10760,21 +10828,21 @@
       <c r="I14" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="J14" s="61"/>
-      <c r="K14" s="61"/>
-      <c r="L14" s="61"/>
-      <c r="M14" s="61"/>
+      <c r="J14" s="62"/>
+      <c r="K14" s="62"/>
+      <c r="L14" s="62"/>
+      <c r="M14" s="62"/>
       <c r="N14" s="51">
         <v>1</v>
       </c>
-      <c r="O14" s="63"/>
-      <c r="P14" s="61"/>
-      <c r="Q14" s="73"/>
+      <c r="O14" s="64"/>
+      <c r="P14" s="62"/>
+      <c r="Q14" s="67"/>
     </row>
     <row r="15" spans="2:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="B15" s="67"/>
-      <c r="C15" s="65"/>
-      <c r="D15" s="69"/>
+      <c r="B15" s="72"/>
+      <c r="C15" s="69"/>
+      <c r="D15" s="75"/>
       <c r="E15" s="24" t="s">
         <v>57</v>
       </c>
@@ -10790,16 +10858,16 @@
       <c r="I15" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="J15" s="65"/>
-      <c r="K15" s="65"/>
-      <c r="L15" s="65"/>
-      <c r="M15" s="65"/>
+      <c r="J15" s="69"/>
+      <c r="K15" s="69"/>
+      <c r="L15" s="69"/>
+      <c r="M15" s="69"/>
       <c r="N15" s="52">
         <v>1</v>
       </c>
-      <c r="O15" s="71"/>
-      <c r="P15" s="65"/>
-      <c r="Q15" s="75"/>
+      <c r="O15" s="76"/>
+      <c r="P15" s="69"/>
+      <c r="Q15" s="68"/>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.6">
       <c r="B20" s="54" t="s">
@@ -10809,6 +10877,19 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="L3:L5"/>
+    <mergeCell ref="L6:L12"/>
+    <mergeCell ref="P3:P5"/>
+    <mergeCell ref="M6:M12"/>
+    <mergeCell ref="P6:P12"/>
+    <mergeCell ref="M3:M5"/>
+    <mergeCell ref="O3:O5"/>
+    <mergeCell ref="O6:O12"/>
+    <mergeCell ref="C6:C12"/>
+    <mergeCell ref="D6:D12"/>
+    <mergeCell ref="J6:J12"/>
+    <mergeCell ref="K6:K12"/>
+    <mergeCell ref="G6:G12"/>
     <mergeCell ref="Q3:Q15"/>
     <mergeCell ref="L13:L15"/>
     <mergeCell ref="M13:M15"/>
@@ -10825,19 +10906,6 @@
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="K3:K5"/>
     <mergeCell ref="B6:B12"/>
-    <mergeCell ref="C6:C12"/>
-    <mergeCell ref="D6:D12"/>
-    <mergeCell ref="J6:J12"/>
-    <mergeCell ref="K6:K12"/>
-    <mergeCell ref="G6:G12"/>
-    <mergeCell ref="L3:L5"/>
-    <mergeCell ref="L6:L12"/>
-    <mergeCell ref="P3:P5"/>
-    <mergeCell ref="M6:M12"/>
-    <mergeCell ref="P6:P12"/>
-    <mergeCell ref="M3:M5"/>
-    <mergeCell ref="O3:O5"/>
-    <mergeCell ref="O6:O12"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10895,7 +10963,7 @@
       <c r="B4" s="17">
         <v>2</v>
       </c>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="79" t="s">
         <v>77</v>
       </c>
       <c r="D4" s="8">
@@ -10911,7 +10979,7 @@
       <c r="B5" s="17">
         <v>3</v>
       </c>
-      <c r="C5" s="70"/>
+      <c r="C5" s="79"/>
       <c r="D5" s="8">
         <v>2.5</v>
       </c>
@@ -10925,7 +10993,7 @@
       <c r="B6" s="17">
         <v>4</v>
       </c>
-      <c r="C6" s="70"/>
+      <c r="C6" s="79"/>
       <c r="D6" s="8">
         <v>7</v>
       </c>
@@ -10939,7 +11007,7 @@
       <c r="B7" s="17">
         <v>5</v>
       </c>
-      <c r="C7" s="70"/>
+      <c r="C7" s="79"/>
       <c r="D7" s="8">
         <v>8</v>
       </c>
@@ -10953,7 +11021,7 @@
       <c r="B8" s="17">
         <v>6</v>
       </c>
-      <c r="C8" s="70"/>
+      <c r="C8" s="79"/>
       <c r="D8" s="8">
         <v>16</v>
       </c>

</xml_diff>